<commit_message>
EN-1264 v0.6 - Zebra auf HKV/Verifikation/Konstanten; Bewertungsspalten erhalten Zebra
- Zebra-Streifen jetzt auch auf HKV-Liste, Verifikation und Konstanten (zebra()-Helfer)
- Auslegung: Bewertungsspalten (rot/gruener Text) bekommen nun das Zebra - Schriftfarbe
  und Streifen in einer kombinierten CF-Regel (vorher verdraengte die Schriftfarbe den Streifen)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FBH_Auslegung_EN1264.xlsx
+++ b/FBH_Auslegung_EN1264.xlsx
@@ -30,7 +30,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Anleitung'!$A$1:$D$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Methodik'!$A$1:$F$26</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Konstanten'!$A$1:$L$28</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Changelog'!$A$1:$C$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -699,13 +699,35 @@
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="6">
+    <dxf>
+      <font>
+        <color rgb="00D32F2F"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0E0E0"/>
+          <bgColor rgb="FFE0E0E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="001E8E1E"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE0E0E0"/>
+          <bgColor rgb="FFE0E0E0"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="00D32F2F"/>
@@ -2156,7 +2178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2183,7 +2205,7 @@
       <c r="B3" s="2" t="n"/>
       <c r="C3" s="21" t="inlineStr">
         <is>
-          <t>Version 0.5 · dh</t>
+          <t>Version 0.6 · dh</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2234,7 @@
     <row r="6">
       <c r="A6" s="108" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="B6" s="109" t="inlineStr">
@@ -2222,7 +2244,7 @@
       </c>
       <c r="C6" s="110" t="inlineStr">
         <is>
-          <t>• Färbung getauscht: berechnete Zellen jetzt mit leichtem grauen Hintergrund, Eingabezellen weiß (alle Blätter).</t>
+          <t>• Zebra-Streifen jetzt auch auf den Blättern HKV, Verifikation und Konstanten.</t>
         </is>
       </c>
     </row>
@@ -2231,33 +2253,33 @@
       <c r="B7" s="111" t="n"/>
       <c r="C7" s="110" t="inlineStr">
         <is>
+          <t>• Auslegung: Bewertungsspalten (rot/grüner Text) erhalten nun tatsächlich das Zebra – Schriftfarbe und Streifen werden in einer kombinierten Regel gesetzt (vorher hat die Schriftfarbe-Regel den Streifen verdrängt).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="108" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="B8" s="109" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C8" s="110" t="inlineStr">
+        <is>
+          <t>• Färbung getauscht: berechnete Zellen jetzt mit leichtem grauen Hintergrund, Eingabezellen weiß (alle Blätter).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="112" t="n"/>
+      <c r="B9" s="112" t="n"/>
+      <c r="C9" s="110" t="inlineStr">
+        <is>
           <t>• Tabellenköpfe durchgehend einheitlich grau (auch Verifikation) – keine weiße Schrift mehr, kein Unterschied zwischen Eingabe- und Rechenspalten im Kopf.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="112" t="n"/>
-      <c r="B8" s="112" t="n"/>
-      <c r="C8" s="110" t="inlineStr">
-        <is>
-          <t>• Bewertungs-Schriftfarben kräftiger (grün/rot); Zebra-Streifen gelten auch für die Bewertungsspalten (rot/grüner Text).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="108" t="inlineStr">
-        <is>
-          <t>0.4</t>
-        </is>
-      </c>
-      <c r="B9" s="109" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="C9" s="110" t="inlineStr">
-        <is>
-          <t>• Graustufen-Design auf ALLE Blätter übertragen: dunkelblaue Flächen/Schrift → Grau bzw. Schwarz, gelbe Eingabefelder → helles Grau.</t>
         </is>
       </c>
     </row>
@@ -2266,33 +2288,33 @@
       <c r="B10" s="111" t="n"/>
       <c r="C10" s="110" t="inlineStr">
         <is>
+          <t>• Bewertungs-Schriftfarben kräftiger (grün/rot); Zebra-Streifen gelten auch für die Bewertungsspalten (rot/grüner Text).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="108" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="B11" s="109" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C11" s="110" t="inlineStr">
+        <is>
+          <t>• Graustufen-Design auf ALLE Blätter übertragen: dunkelblaue Flächen/Schrift → Grau bzw. Schwarz, gelbe Eingabefelder → helles Grau.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="112" t="n"/>
+      <c r="B12" s="112" t="n"/>
+      <c r="C12" s="110" t="inlineStr">
+        <is>
           <t>• Auslegung: Status-Spalte (✓/!) wieder entfernt; Bewertung jetzt über die Schriftfarbe – leicht grün = im Rahmen, leicht rot = Grenzwert überschritten (auch in Kontrolle und Verifikation).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="112" t="n"/>
-      <c r="B11" s="112" t="n"/>
-      <c r="C11" s="110" t="inlineStr">
-        <is>
-          <t>• Tabellenkopf einheitlich in kräftigerem Grau; editierbare Zellen in hellerem Grau.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="108" t="inlineStr">
-        <is>
-          <t>0.3</t>
-        </is>
-      </c>
-      <c r="B12" s="109" t="inlineStr">
-        <is>
-          <t>2026-06-17</t>
-        </is>
-      </c>
-      <c r="C12" s="110" t="inlineStr">
-        <is>
-          <t>• Diese EN-1264-Mappe ist jetzt die Hauptvariante; die vereinfachte Mappe wurde nach 'archiv/' verschoben.</t>
         </is>
       </c>
     </row>
@@ -2301,16 +2323,24 @@
       <c r="B13" s="111" t="n"/>
       <c r="C13" s="110" t="inlineStr">
         <is>
-          <t>• Auslegung im Graustufen-Design: Schrift durchgehend schwarz (auch Einheiten), Eingabe-/editierbare Zellen grau hinterlegt; Farbe nur noch im Logo.</t>
+          <t>• Tabellenkopf einheitlich in kräftigerem Grau; editierbare Zellen in hellerem Grau.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="111" t="n"/>
-      <c r="B14" s="111" t="n"/>
+      <c r="A14" s="108" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="B14" s="109" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
       <c r="C14" s="110" t="inlineStr">
         <is>
-          <t>• Bewertung als Symbol statt Farbe: neue Spalte 'Status' mit ✓ (alle Prüfungen ok) bzw. ! (Warnung) – auch im Schwarz-Weiß-Druck erkennbar; rote/grüne Zellhintergründe entfallen.</t>
+          <t>• Diese EN-1264-Mappe ist jetzt die Hauptvariante; die vereinfachte Mappe wurde nach 'archiv/' verschoben.</t>
         </is>
       </c>
     </row>
@@ -2319,24 +2349,16 @@
       <c r="B15" s="112" t="n"/>
       <c r="C15" s="110" t="inlineStr">
         <is>
-          <t>• Zebra-Streifen (jede zweite sichtbare Zeile) über bedingte Formatierung mit SUBTOTAL (filterfest); neue Filterfunktion (AutoFilter), Filtern trotz Blattschutz möglich.</t>
+          <t>• Auslegung im Graustufen-Design: Schrift durchgehend schwarz (auch Einheiten), Eingabe-/editierbare Zellen grau hinterlegt; Farbe nur noch im Logo.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="108" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
-      </c>
-      <c r="B16" s="109" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
+      <c r="A16" s="112" t="n"/>
+      <c r="B16" s="112" t="n"/>
       <c r="C16" s="110" t="inlineStr">
         <is>
-          <t>• EN-1264-Parameter (B, a_ü, a_D, m_ü, m_D) von den Grundeinstellungen ins Blatt 'Konstanten' verschoben – alle EN-1264-Faktoren stehen jetzt zusammen.</t>
+          <t>• Bewertung als Symbol statt Farbe: neue Spalte 'Status' mit ✓ (alle Prüfungen ok) bzw. ! (Warnung) – auch im Schwarz-Weiß-Druck erkennbar; rote/grüne Zellhintergründe entfallen.</t>
         </is>
       </c>
     </row>
@@ -2345,33 +2367,33 @@
       <c r="B17" s="111" t="n"/>
       <c r="C17" s="110" t="inlineStr">
         <is>
+          <t>• Zebra-Streifen (jede zweite sichtbare Zeile) über bedingte Formatierung mit SUBTOTAL (filterfest); neue Filterfunktion (AutoFilter), Filtern trotz Blattschutz möglich.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="108" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="B18" s="109" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C18" s="110" t="inlineStr">
+        <is>
+          <t>• EN-1264-Parameter (B, a_ü, a_D, m_ü, m_D) von den Grundeinstellungen ins Blatt 'Konstanten' verschoben – alle EN-1264-Faktoren stehen jetzt zusammen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="112" t="n"/>
+      <c r="B19" s="112" t="n"/>
+      <c r="C19" s="110" t="inlineStr">
+        <is>
           <t>• Konstanten neu geordnet: jede Tabelle durch weiße Leerzellen/-spalten optisch getrennt; passt auf eine A4-Quer-Seite.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="112" t="n"/>
-      <c r="B18" s="112" t="n"/>
-      <c r="C18" s="110" t="inlineStr">
-        <is>
-          <t>• Verifikation/Hinweise sprachlich bereinigt (kein Verweis mehr auf einen Systemfaktor; Faktor-Werte können durch die Norm-Werte ersetzt werden).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="108" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="B19" s="109" t="inlineStr">
-        <is>
-          <t>2026-06-16</t>
-        </is>
-      </c>
-      <c r="C19" s="110" t="inlineStr">
-        <is>
-          <t>• Eigenständige Mappe: vollständige Auslegung nach dem Berechnungsansatz der DIN EN 1264-2 (Bauart A, Heizrohre im Estrich).</t>
         </is>
       </c>
     </row>
@@ -2380,34 +2402,42 @@
       <c r="B20" s="111" t="n"/>
       <c r="C20" s="110" t="inlineStr">
         <is>
+          <t>• Verifikation/Hinweise sprachlich bereinigt (kein Verweis mehr auf einen Systemfaktor; Faktor-Werte können durch die Norm-Werte ersetzt werden).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="108" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="B21" s="109" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C21" s="110" t="inlineStr">
+        <is>
+          <t>• Eigenständige Mappe: vollständige Auslegung nach dem Berechnungsansatz der DIN EN 1264-2 (Bauart A, Heizrohre im Estrich).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="112" t="n"/>
+      <c r="B22" s="112" t="n"/>
+      <c r="C22" s="110" t="inlineStr">
+        <is>
           <t>• Wärmestromdichte über das Produktverfahren q = B · a_B · a_T^mT · a_ü^mü · a_D^mD · ΔθH (kein pauschaler Systemfaktor f mehr).</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="111" t="n"/>
-      <c r="B21" s="111" t="n"/>
-      <c r="C21" s="110" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="112" t="n"/>
+      <c r="B23" s="112" t="n"/>
+      <c r="C23" s="110" t="inlineStr">
         <is>
           <t>• Faktoren a_B(R) und a_T(R) als editierbare Tabelle (an die veröffentlichten EN-1264-Leistungstabellen kalibriert: fbh24 max. 1,2 %, Rehau 17×2 −1,7 % gesamt).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="111" t="n"/>
-      <c r="B22" s="111" t="n"/>
-      <c r="C22" s="110" t="inlineStr">
-        <is>
-          <t>• Exponenten m_T = 1 − Verlegeabstand/0,075, m_ü = 100·(0,045 − s_ü), m_D = 250·(D − 0,020) aus den Geometriedaten; Systemkoeffizient B = 6,7 W/m²K.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="111" t="n"/>
-      <c r="B23" s="111" t="n"/>
-      <c r="C23" s="110" t="inlineStr">
-        <is>
-          <t>• Hydraulik (Massenstrom, Druckverlust nach Darcy-Weisbach), HKV-Auswertung und Kontrolle wie im vereinfachten Tool.</t>
         </is>
       </c>
     </row>
@@ -2416,23 +2446,43 @@
       <c r="B24" s="112" t="n"/>
       <c r="C24" s="110" t="inlineStr">
         <is>
+          <t>• Exponenten m_T = 1 − Verlegeabstand/0,075, m_ü = 100·(0,045 − s_ü), m_D = 250·(D − 0,020) aus den Geometriedaten; Systemkoeffizient B = 6,7 W/m²K.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="112" t="n"/>
+      <c r="B25" s="112" t="n"/>
+      <c r="C25" s="110" t="inlineStr">
+        <is>
+          <t>• Hydraulik (Massenstrom, Druckverlust nach Darcy-Weisbach), HKV-Auswertung und Kontrolle wie im vereinfachten Tool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="111" t="n"/>
+      <c r="B26" s="111" t="n"/>
+      <c r="C26" s="110" t="inlineStr">
+        <is>
           <t>• Hinweis: a_B/a_T sind kalibriert, a_ü/a_D EN-1264-orientierte Richtwerte – bei Bedarf gegen die Norm-Tabelle (DIN EN 1264-2, Tab. A.1) prüfen.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
-  <mergeCells count="10">
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="A12:A15"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="B12:B15"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="B19:B24"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="A19:A24"/>
-    <mergeCell ref="A6:A8"/>
-    <mergeCell ref="B6:B8"/>
+  <mergeCells count="12">
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A21:A26"/>
+    <mergeCell ref="B21:B26"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A18:A20"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -27382,72 +27432,114 @@
   </mergeCells>
   <conditionalFormatting sqref="R7:R206">
     <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(AND($R7&lt;&gt;"",$R7&gt;$S7),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>AND(AND($R7&lt;&gt;"",$R7&lt;=$S7),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
       <formula>AND($R7&lt;&gt;"",$R7&gt;$S7)</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="4" dxfId="3">
       <formula>AND($R7&lt;&gt;"",$R7&lt;=$S7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T7:T206">
-    <cfRule type="expression" priority="3" dxfId="0">
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>AND(AND($T7&lt;&gt;"",$F7&lt;&gt;"",$T7&lt;$F7),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="1">
+      <formula>AND(AND($T7&lt;&gt;"",$F7&lt;&gt;"",$T7&gt;=$F7),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="2">
       <formula>AND($T7&lt;&gt;"",$F7&lt;&gt;"",$T7&lt;$F7)</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="1">
+    <cfRule type="expression" priority="8" dxfId="3">
       <formula>AND($T7&lt;&gt;"",$F7&lt;&gt;"",$T7&gt;=$F7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V7:V206">
-    <cfRule type="expression" priority="5" dxfId="0">
+    <cfRule type="expression" priority="9" dxfId="0">
+      <formula>AND(AND($V7&lt;&gt;"",$V7&lt;1),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="1">
+      <formula>AND(AND($V7&lt;&gt;"",$V7&gt;=1),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="2">
       <formula>AND($V7&lt;&gt;"",$V7&lt;1)</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="1">
+    <cfRule type="expression" priority="12" dxfId="3">
       <formula>AND($V7&lt;&gt;"",$V7&gt;=1)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB7:AB206">
-    <cfRule type="expression" priority="7" dxfId="0">
+    <cfRule type="expression" priority="13" dxfId="0">
+      <formula>AND(AND($AB7&lt;&gt;"",$AB7&gt;'Grundeinstellungen'!$C$11),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="1">
+      <formula>AND(AND($AB7&lt;&gt;"",$AB7&lt;='Grundeinstellungen'!$C$11),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="2">
       <formula>AND($AB7&lt;&gt;"",$AB7&gt;'Grundeinstellungen'!$C$11)</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="1">
+    <cfRule type="expression" priority="16" dxfId="3">
       <formula>AND($AB7&lt;&gt;"",$AB7&lt;='Grundeinstellungen'!$C$11)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD7:AD206">
-    <cfRule type="expression" priority="9" dxfId="0">
+    <cfRule type="expression" priority="17" dxfId="0">
+      <formula>AND(AND($AD7&lt;&gt;"",$AD7&gt;'Grundeinstellungen'!$C$22),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="1">
+      <formula>AND(AND($AD7&lt;&gt;"",$AD7&lt;='Grundeinstellungen'!$C$22),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="19" dxfId="2">
       <formula>AND($AD7&lt;&gt;"",$AD7&gt;'Grundeinstellungen'!$C$22)</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" dxfId="1">
+    <cfRule type="expression" priority="20" dxfId="3">
       <formula>AND($AD7&lt;&gt;"",$AD7&lt;='Grundeinstellungen'!$C$22)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK7:AK206">
-    <cfRule type="expression" priority="11" dxfId="0">
+    <cfRule type="expression" priority="21" dxfId="0">
+      <formula>AND(AND($AK7&lt;&gt;"",$AK7&gt;'Grundeinstellungen'!$C$12),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="22" dxfId="1">
+      <formula>AND(AND($AK7&lt;&gt;"",$AK7&lt;='Grundeinstellungen'!$C$12),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="23" dxfId="2">
       <formula>AND($AK7&lt;&gt;"",$AK7&gt;'Grundeinstellungen'!$C$12)</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" dxfId="1">
+    <cfRule type="expression" priority="24" dxfId="3">
       <formula>AND($AK7&lt;&gt;"",$AK7&lt;='Grundeinstellungen'!$C$12)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE7:AE206">
-    <cfRule type="expression" priority="13" dxfId="0">
+    <cfRule type="expression" priority="25" dxfId="0">
+      <formula>AND(AND($AE7&lt;&gt;"",OR($AE7&lt;'Grundeinstellungen'!$C$20,$AE7&gt;'Grundeinstellungen'!$C$21)),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="26" dxfId="1">
+      <formula>AND(AND($AE7&lt;&gt;"",$AE7&gt;='Grundeinstellungen'!$C$20,$AE7&lt;='Grundeinstellungen'!$C$21),MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="27" dxfId="2">
       <formula>AND($AE7&lt;&gt;"",OR($AE7&lt;'Grundeinstellungen'!$C$20,$AE7&gt;'Grundeinstellungen'!$C$21))</formula>
     </cfRule>
-    <cfRule type="expression" priority="14" dxfId="1">
+    <cfRule type="expression" priority="28" dxfId="3">
       <formula>AND($AE7&lt;&gt;"",$AE7&gt;='Grundeinstellungen'!$C$20,$AE7&lt;='Grundeinstellungen'!$C$21)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H7:H206">
-    <cfRule type="expression" priority="15" dxfId="0">
+    <cfRule type="expression" priority="29" dxfId="2">
       <formula>AND($H7&lt;&gt;"",$D7&lt;&gt;"",$H7&gt;$D7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A7:A206 B7:B206 C7:C206 D7:D206 E7:E206 F7:F206 H7:H206 I7:I206 J7:J206 K7:K206 L7:L206 M7:M206">
-    <cfRule type="expression" priority="16" dxfId="2">
+    <cfRule type="expression" priority="30" dxfId="4">
       <formula>AND($B7&lt;&gt;"",MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G7:G206 N7:N206 O7:O206 P7:P206 Q7:Q206 R7:R206 S7:S206 T7:T206 U7:U206 V7:V206 W7:W206 X7:X206 Y7:Y206 Z7:Z206 AA7:AA206 AB7:AB206 AC7:AC206 AD7:AD206 AE7:AE206 AF7:AF206 AG7:AG206 AH7:AH206 AI7:AI206 AJ7:AJ206 AK7:AK206">
-    <cfRule type="expression" priority="17" dxfId="3">
+  <conditionalFormatting sqref="G7:G206 N7:N206 O7:O206 P7:P206 Q7:Q206 S7:S206 U7:U206 W7:W206 X7:X206 Y7:Y206 Z7:Z206 AA7:AA206 AC7:AC206 AF7:AF206 AG7:AG206 AH7:AH206 AI7:AI206 AJ7:AJ206">
+    <cfRule type="expression" priority="31" dxfId="5">
       <formula>AND($B7&lt;&gt;"",MOD(SUBTOTAL(103,$B$7:$B7),2)=0)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -27876,50 +27968,50 @@
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <conditionalFormatting sqref="B20">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="2">
       <formula>$B$20&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="2" dxfId="3">
       <formula>$B$20=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B21">
-    <cfRule type="expression" priority="3" dxfId="0">
+    <cfRule type="expression" priority="3" dxfId="2">
       <formula>$B$21&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="1">
+    <cfRule type="expression" priority="4" dxfId="3">
       <formula>$B$21=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22">
-    <cfRule type="expression" priority="5" dxfId="0">
+    <cfRule type="expression" priority="5" dxfId="2">
       <formula>$B$22&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="1">
+    <cfRule type="expression" priority="6" dxfId="3">
       <formula>$B$22=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B23">
-    <cfRule type="expression" priority="7" dxfId="0">
+    <cfRule type="expression" priority="7" dxfId="2">
       <formula>$B$23&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="1">
+    <cfRule type="expression" priority="8" dxfId="3">
       <formula>$B$23=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
-    <cfRule type="expression" priority="9" dxfId="0">
+    <cfRule type="expression" priority="9" dxfId="2">
       <formula>$B$24&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" dxfId="1">
+    <cfRule type="expression" priority="10" dxfId="3">
       <formula>$B$24=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B25">
-    <cfRule type="expression" priority="11" dxfId="0">
+    <cfRule type="expression" priority="11" dxfId="2">
       <formula>$B$25&gt;0</formula>
     </cfRule>
-    <cfRule type="expression" priority="12" dxfId="1">
+    <cfRule type="expression" priority="12" dxfId="3">
       <formula>$B$25=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -29769,6 +29861,11 @@
   <mergeCells count="1">
     <mergeCell ref="F2:G2"/>
   </mergeCells>
+  <conditionalFormatting sqref="A5:H54">
+    <cfRule type="expression" priority="1" dxfId="5">
+      <formula>AND($A5&lt;&gt;"",MOD(SUBTOTAL(103,$A$5:$A5),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -30670,17 +30767,53 @@
   </mergeCells>
   <conditionalFormatting sqref="I9:I20">
     <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(AND($I9&lt;&gt;"",ABS($I9)&gt;0.05),MOD(SUBTOTAL(103,$A$9:$A9),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>AND(AND($I9&lt;&gt;"",ABS($I9)&lt;=0.05),MOD(SUBTOTAL(103,$A$9:$A9),2)=0)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
       <formula>AND($I9&lt;&gt;"",ABS($I9)&gt;0.05)</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="4" dxfId="3">
       <formula>AND($I9&lt;&gt;"",ABS($I9)&lt;=0.05)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A9:F20">
+    <cfRule type="expression" priority="5" dxfId="4">
+      <formula>AND($A9&lt;&gt;"",MOD(SUBTOTAL(103,$A$9:$A9),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9:G20">
+    <cfRule type="expression" priority="6" dxfId="5">
+      <formula>AND($A9&lt;&gt;"",MOD(SUBTOTAL(103,$A$9:$A9),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H9:H20">
+    <cfRule type="expression" priority="7" dxfId="5">
+      <formula>AND($A9&lt;&gt;"",MOD(SUBTOTAL(103,$A$9:$A9),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J9:J20">
+    <cfRule type="expression" priority="8" dxfId="5">
+      <formula>AND($A9&lt;&gt;"",MOD(SUBTOTAL(103,$A$9:$A9),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K9:K20">
+    <cfRule type="expression" priority="9" dxfId="5">
+      <formula>AND($A9&lt;&gt;"",MOD(SUBTOTAL(103,$A$9:$A9),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L9:L20">
+    <cfRule type="expression" priority="10" dxfId="5">
+      <formula>AND($A9&lt;&gt;"",MOD(SUBTOTAL(103,$A$9:$A9),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I21">
-    <cfRule type="expression" priority="3" dxfId="0">
+    <cfRule type="expression" priority="11" dxfId="2">
       <formula>AND($I21&lt;&gt;"",ABS($I21)&gt;0.05)</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="1">
+    <cfRule type="expression" priority="12" dxfId="3">
       <formula>AND($I21&lt;&gt;"",ABS($I21)&lt;=0.05)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -32553,6 +32686,26 @@
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A4:C4"/>
   </mergeCells>
+  <conditionalFormatting sqref="A6:C10">
+    <cfRule type="expression" priority="1" dxfId="4">
+      <formula>AND($A6&lt;&gt;"",MOD(SUBTOTAL(103,$A$6:$A6),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A21:E28">
+    <cfRule type="expression" priority="2" dxfId="4">
+      <formula>AND($A21&lt;&gt;"",MOD(SUBTOTAL(103,$A$21:$A21),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G6:I13">
+    <cfRule type="expression" priority="3" dxfId="4">
+      <formula>AND($G6&lt;&gt;"",MOD(SUBTOTAL(103,$G$6:$G6),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K6:L25">
+    <cfRule type="expression" priority="4" dxfId="4">
+      <formula>AND($K6&lt;&gt;"",MOD(SUBTOTAL(103,$K$6:$K6),2)=0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <headerFooter>

</xml_diff>